<commit_message>
Add reusable 'cod-market-analysis' skill: full Alibaba-links -> Arabic study pipeline
SKILL.md workflow (identify -> keywords -> Meta Ad Library hunt -> competitors/links/creatives ->
pricing/margin -> risk -> Arabic reports -> Excel + recommendation + PDFs), plus references
(hunter_protocol, report template, JSON schemas) and generalized build scripts (CSV, XLSX, links
annex PDF, consolidated study PDF) that take the analysis folder as arg and auto-render Arabic RTL
PDFs via Chromium. Verified end-to-end against the Libya dataset. Adds data/study_meta.json example.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ETY9xkuviAkpRZEz8Cpsma
</commit_message>
<xml_diff>
--- a/libya-market-analysis/مقارنة_المنتجات.xlsx
+++ b/libya-market-analysis/مقارنة_المنتجات.xlsx
@@ -28,10 +28,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -41,11 +40,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C05621"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0F0F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -90,9 +84,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -101,13 +98,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,20 +471,20 @@
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46" customHeight="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>المنتج</t>
@@ -516,7 +507,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>إجمالي الإعلانات المرصودة</t>
+          <t>إجمالي الإعلانات</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -526,27 +517,27 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>إعلانات طويلة العمر (&gt;60 يوم)</t>
+          <t>إعلانات &gt;60 يوم</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>سعر البيع الليبي المرصود (د.ل)</t>
+          <t>سعر ليبي مرصود (د.ل)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>تكلفة+شحن الوحدة (تقدير)</t>
+          <t>تكلفة+شحن</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>الهامش/طلب مُسلَّم (تقدير)</t>
+          <t>الهامش/طلب مُسلَّم</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>أعلى درجة خطر</t>
+          <t>أعلى خطر</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -563,7 +554,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>منتج AliExpress غير محدد</t>
+          <t>aliexpress unknown</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -616,102 +607,102 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>مشد نسائي (شيبروير)</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>shapewear</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>P02</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="F3" s="4" t="n">
-        <v>547</v>
-      </c>
-      <c r="G3" s="4" t="n">
+      <c r="F3" s="2" t="n">
+        <v>548</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>51</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>≈ 2–5 دولار للوحدة (فئة) + شحن جوي ≈ 0.5–1 دولار ⇒ ≈ 21–51 د.ل (موازي)</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>سعر بيع ليبي مرصود 51 د.ل؛ سعر مقترح 79–99 د.ل ⇒ هامش خام ≈ 40–70 د.ل، وبعد احتساب ≈50% تسليم ≈ 20–35 د.ل/طلب مؤكد</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>16/25 (تشبّع السوق + إجهاد الإعلانات)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="L3" s="4" t="n">
         <v>6.5</v>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>طلب مثبت وقوي (QAVA 40 إعلان، Liposta 77، BaraBora مستمر منذ يناير 2025) لكن السوق مشبع عالمياً ومخاطر إرجاع المقاسات مرتفعة تحت COD.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>جهاز ألتراسونيك منزلي (مرطب/فواحة)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ultrasonic device</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>P03</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="F4" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="G4" s="4" t="n">
+      <c r="F4" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>غير متوفر</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>≈ 3–8 دولار للوحدة (فئة) + شحن ⇒ ≈ 30–75 د.ل (تقدير)</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>غير متوفر بدقة — لا سعر بيع ليبي مرصود؛ تقدير هامش متوسط إن بيع بـ 99–149 د.ل</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>16/25 (غموض هوية المنتج + سوق ضحل)</t>
         </is>
@@ -719,219 +710,219 @@
       <c r="L4" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>سوق ضحل: 4 منافسين فقط. القراءة المدعومة محلياً هي المرطّب/الفوّاحة العطرية وليست منظّف الألتراسونيك (كل مصطلحات المنظّف رجعت صفراً).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>قلادة ذهبية هدية للأم</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>gold necklace gift</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>P04</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="F5" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>21، 150</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>≈ 1–3 دولار للوحدة (مطلية) + شحن جوي ≈ 0.3–0.8 دولار ⇒ ≈ 11–32 د.ل (موازي)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>أسعار ليبية مرصودة 21 د.ل (قطعة) و150 د.ل (طقم هدية)؛ سعر مقترح 99–149 د.ل ⇒ هامش خام ≈ 70–130 د.ل، وبعد ≈50% تسليم ≈ 35–65 د.ل/طلب مؤكد</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>12/25 (منافسة نشطة على المصطلحات العامة)</t>
         </is>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="L5" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>أعلى نشاط إعلاني على الإطلاق: ليبيا إكسبريس 187 إعلاناً نشطاً، Libya Express 72، 4F Badia 58. طلب هدايا مُثبت وضخم، وحدة خفيفة رخيصة، مقاس عالمي = إرجاع منخفض.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>قلادة ماما</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>mama necklace</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>P05</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="G6" s="4" t="n">
+      <c r="F6" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>≈ 1–3 دولار للوحدة + شحن ⇒ ≈ 11–32 د.ل (موازي)</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>سعر ليبي مرصود 21 د.ل؛ سعر مقترح 89–129 د.ل ⇒ هامش خام مرتفع نظرياً، لكن الطلب على النقش «ماما» تحديداً غير مُثبت</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>12/25 (طلب المتغيّر المحدد غير مُثبت)</t>
         </is>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="L6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>لا يوجد أي معلن ليبي يروّج قلادة نقش «ماما» تحديداً (كل المصطلحات المخصصة رجعت صفراً)؛ الطلب المشترك يأتي من صفحات هدايا القلادات نفسها في P04.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>فرشاة أسنان كهربائية للأطفال حرف U</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>kids u toothbrush</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>P06</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>127</v>
-      </c>
-      <c r="G7" s="4" t="n">
+      <c r="F7" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>≈ 5.4–14 دولار للوحدة (فئة) + شحن ⇒ ≈ 50–130 د.ل (تقدير)</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>سعر ليبي مرصود 75 د.ل؛ سعر مقترح 99–149 د.ل ⇒ هامش متوسط، وبطارية = قيد شحن</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>16/25 (جودة/إرجاع + سلامة الأطفال)</t>
         </is>
       </c>
-      <c r="L7" s="5" t="n">
+      <c r="L7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>طلب متوسط عبر متاجر عامة: لحظة-Momento 36 إعلاناً منذ 2026-03-04 (طويلة الأمد)، NajdMarket 20. منتج أطفال حسّاس للجودة.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>جهاز عمل الآيس كريم رول</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ice cream maker</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>P07</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="F8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G8" s="4" t="n">
+      <c r="F8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>غير متوفر</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>غموض فئة: عدّة رخيصة ≈ 3–10$ مقابل ماكينة تجارية 739$+ ⇒ التكلفة غير محسومة</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>غير متوفر بدقة — لا سعر بيع ليبي مرصود؛ المنتج موسمي وضخم/هش</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>16/25 (موسمية + هشاشة/حجم الشحن)</t>
         </is>
@@ -939,109 +930,109 @@
       <c r="L8" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>سوق ضحل جداً: منافسان فقط ذوا صلة. غموض في فئة المنتج (عدّة منزلية رخيصة أم ماكينة تجارية) وموسمية صيفية وحجم شحن كبير.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>قفل مقبض الباب للحماية</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>door lever lock</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>P08</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>272</v>
-      </c>
-      <c r="G9" s="4" t="n">
+      <c r="F9" s="2" t="n">
+        <v>273</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>غير متوفر</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>≈ 3.86–9.99 دولار للوحدة (فئة أقفال مشابهة) + شحن ⇒ ≈ 33–85 د.ل (تقدير)</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>غير متوفر بدقة — لا سعر بيع ليبي مرصود؛ لكن عمق إعلاني جيد على أقفال الأمان</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>12/25 (عدم تطابق هوية: مقبض مقابل قفل أمان أطفال)</t>
         </is>
       </c>
-      <c r="L9" s="5" t="n">
+      <c r="L9" s="4" t="n">
         <v>5.5</v>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>عمق إعلاني جيد على أقفال الأمان: سوقنا 39 إعلاناً، Souq tika مستمر منذ 2025-10-10، lock factory 16. لكن ما يُباع فعلاً هو أقفال أمان الأطفال، وقد يختلف عن «قفل المقبض» المصدر.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>طاولة/أباجورة سرير قابلة للطي</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>bedside table lamp</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>P09</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>485</v>
-      </c>
-      <c r="G10" s="4" t="n">
+      <c r="F10" s="2" t="n">
+        <v>486</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>≈ 13–71 دولار (فئة أثاث/إضاءة) + شحن حجمي ⇒ مرتفع نسبياً</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>سعر ليبي مرصود 62 د.ل؛ لكن السوق ضحل والوحدة أثقل/أكبر</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>16/25 (هشاشة/حجم الشحن + كهرباء)</t>
         </is>
@@ -1049,54 +1040,54 @@
       <c r="L10" s="3" t="n">
         <v>4.5</v>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>سوق نظيف لكنه ضحل: 5 منافسين و5 إعلانات فقط، لا منافس مخصّص. Diollo Store (34 إعلاناً منذ 2025-07) متجر أدوات عام. وحدة أثقل/كهربائية.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>قفازات الشواء المقاومة للحرارة</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>bbq gloves</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="G11" s="4" t="n">
+      <c r="F11" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>غير متوفر</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>غير متوفر (لا سعر بيع ليبي) — الوحدة رخيصة لكن لا سوق</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>غير متوفر — لا طلب مُثبت في ليبيا</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>12/25 (لكن الخطر الأكبر: غياب الطلب أصلاً)</t>
         </is>
@@ -1104,54 +1095,54 @@
       <c r="L11" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>النيتش فارغ فعلياً في ليبيا: 11 من 12 كلمة مفتاحية رجعت صفر إعلان، والنتيجة الوحيدة إعلان خارج الموضوع. لا طلب مُثبت.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>رضّاعة أطفال صديقة للبيئة</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>baby bottle</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>127</v>
-      </c>
-      <c r="G12" s="4" t="n">
+      <c r="F12" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>غير متوفر</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>≈ 0.32–6 دولار (زجاج) / MOQ عالٍ للسيليكون + شحن ⇒ ≈ 3–55 د.ل (تقدير)</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>غير متوفر بدقة — لا سعر بيع ليبي مرصود؛ سوق ضحل ومتاجر تقليدية</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>12/25 (سلامة/جودة منتج رضّع + إرجاع)</t>
         </is>
@@ -1159,62 +1150,62 @@
       <c r="L12" s="3" t="n">
         <v>4.5</v>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>سوق حقيقي لكنه ضحل: 7 صفحات ذات صلة، كلّها متاجر مستلزمات أم وطفل تقليدية بإعلان أو اثنين، لا معلن COD مخصّص لرضّاعة مفردة.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>ماكينة حلاقة نسائية لاسلكية</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>lady shaver</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>446</v>
-      </c>
-      <c r="G13" s="4" t="n">
+      <c r="F13" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>غير متوفر</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>≈ 1.19–5.09 دولار للوحدة (فئة) + شحن ⇒ ≈ 10–43 د.ل (تقدير)</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>غير متوفر بدقة — لا سعر بيع ليبي مرصود للمنتج المحدد؛ لكن فئة إزالة الشعر نشطة</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>16/25 (حساسية COD لمنتج نظافة شخصية + بطارية)</t>
         </is>
       </c>
-      <c r="L13" s="5" t="n">
+      <c r="L13" s="4" t="n">
         <v>5.5</v>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>فئة إزالة الشعر نشطة (ليبيا شوب 94 إعلاناً، ماركة منذ 2025-04) لكن لا أحد يعلن ماكينة الحلاقة النسائية اللاسلكية تحديداً. منتج نظافة شخصية + بطارية.</t>
         </is>

</xml_diff>